<commit_message>
Fix missing section for 23UR section 2
</commit_message>
<xml_diff>
--- a/apps/chodby_inv/input_data/wpt_2025_04_with_flux_on_multipacker.xlsx
+++ b/apps/chodby_inv/input_data/wpt_2025_04_with_flux_on_multipacker.xlsx
@@ -8020,7 +8020,9 @@
       <c r="A281" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B281" s="1"/>
+      <c r="B281" s="1" t="n">
+        <v>2</v>
+      </c>
       <c r="C281" s="1" t="s">
         <v>72</v>
       </c>

</xml_diff>